<commit_message>
update layout, fix problems and config output files
</commit_message>
<xml_diff>
--- a/Project Ouputs/BOM/Bill of Materials-sme-pcb-energysolution-s01.xlsx
+++ b/Project Ouputs/BOM/Bill of Materials-sme-pcb-energysolution-s01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\sme\PCB\sme-pcb-energysolution-s01\Project Ouputs\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9D05EC9-20A1-4E5F-8FCC-3C730481964F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{046D59B9-3DED-43CA-ABD9-52294A7AE2A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="6075" windowWidth="29040" windowHeight="15720" xr2:uid="{897580FB-078F-49CA-9E73-4E0E85F8360C}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C15F647B-C887-43F2-9E13-23750635C920}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-sme-pcb-energ" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="200">
   <si>
     <t>Line #</t>
   </si>
@@ -122,7 +122,7 @@
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 50 V 0.1uF X7R 0603 10%</t>
   </si>
   <si>
-    <t>C6, C9, C10, C14, C18</t>
+    <t>C6, C10, C14, C18</t>
   </si>
   <si>
     <t>603-CC603KRX7R9BB104</t>
@@ -140,6 +140,18 @@
     <t>603-CC603KRX5R6BB105</t>
   </si>
   <si>
+    <t>CC0603KRX7R5BB225</t>
+  </si>
+  <si>
+    <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 6.3V 2.2uF X7R 0603 10% HI CV</t>
+  </si>
+  <si>
+    <t>C9</t>
+  </si>
+  <si>
+    <t>603-CC603KRX7R5BB225</t>
+  </si>
+  <si>
     <t>CDBB240-HF</t>
   </si>
   <si>
@@ -236,7 +248,10 @@
     <t>630-HSMS-C170</t>
   </si>
   <si>
-    <t>XH-2 Connector</t>
+    <t>B2B-XH-AM(LF)(SN)</t>
+  </si>
+  <si>
+    <t>CONN HEADER VERT 2POS 2.5MM</t>
   </si>
   <si>
     <t>P1, P2, P3, P4</t>
@@ -245,10 +260,7 @@
     <t>JST</t>
   </si>
   <si>
-    <t>B2B-XH-2(LF)(SN)</t>
-  </si>
-  <si>
-    <t>306-B2B-XH-2LFSN</t>
+    <t>306-B2B-XH-AMLFSNP</t>
   </si>
   <si>
     <t>N-CH</t>
@@ -338,7 +350,7 @@
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0805, 0Ohms, 1%, 1/8W</t>
   </si>
   <si>
-    <t>R5, R18</t>
+    <t>R5, R15</t>
   </si>
   <si>
     <t>RC0805FR-10100RL</t>
@@ -365,58 +377,58 @@
     <t>Thin Film Resistors - SMD 1M OHM 1% 50PPM 1/10 W</t>
   </si>
   <si>
-    <t>R7, R8, R9, R33</t>
+    <t>R7, R8, R32</t>
   </si>
   <si>
     <t>603-RT0603FRE071ML</t>
   </si>
   <si>
-    <t>RT0603FRD07180KL</t>
-  </si>
-  <si>
-    <t>Thin Film Resistors - SMD 180K OHM 1% 25PPM 1/10W</t>
+    <t>RT0603FRE0720KL</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors - SMD 1/10W 20K ohm 1% 50ppm</t>
+  </si>
+  <si>
+    <t>R9</t>
+  </si>
+  <si>
+    <t>603-RT0603FRE0720KL</t>
+  </si>
+  <si>
+    <t>PE1206FRE470R02L</t>
+  </si>
+  <si>
+    <t>Current Sense Resistors - SMD 20 mOhms 1 W 50PPM/C 1206</t>
   </si>
   <si>
     <t>R10</t>
   </si>
   <si>
-    <t>603-RT0603FRD07180KL</t>
-  </si>
-  <si>
-    <t>RT0603FRE0720KL</t>
-  </si>
-  <si>
-    <t>Thin Film Resistors - SMD 1/10W 20K ohm 1% 50ppm</t>
+    <t>603-PE1206FRE470R02L</t>
+  </si>
+  <si>
+    <t>RT0603FRE0727KL</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors - SMD 1/10W 27K ohm 1% 50ppm</t>
   </si>
   <si>
     <t>R11</t>
   </si>
   <si>
-    <t>603-RT0603FRE0720KL</t>
-  </si>
-  <si>
-    <t>PE1206FRE470R02L</t>
-  </si>
-  <si>
-    <t>Current Sense Resistors - SMD 20 mOhms 1 W 50PPM/C 1206</t>
+    <t>603-RT0603FRE0727KL</t>
+  </si>
+  <si>
+    <t>RT0603FRE072KL</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors - SMD 1/10W 2K ohm 1% 50ppm</t>
   </si>
   <si>
     <t>R12</t>
   </si>
   <si>
-    <t>603-PE1206FRE470R02L</t>
-  </si>
-  <si>
-    <t>RT0603FRE0727KL</t>
-  </si>
-  <si>
-    <t>Thin Film Resistors - SMD 1/10W 27K ohm 1% 50ppm</t>
-  </si>
-  <si>
-    <t>R13, R14</t>
-  </si>
-  <si>
-    <t>603-RT0603FRE0727KL</t>
+    <t>603-RT0603FRE072KL</t>
   </si>
   <si>
     <t>RT0603BRD0732KL</t>
@@ -425,7 +437,7 @@
     <t>Thin Film Resistors - SMD 1/10W 32K Ohms 0.1%</t>
   </si>
   <si>
-    <t>R15, R20</t>
+    <t>R13</t>
   </si>
   <si>
     <t>603-RT0603BRD0732KL</t>
@@ -437,37 +449,58 @@
     <t>Thin Film Resistors - SMD 100K OHM 1% 25PPM 1/10W</t>
   </si>
   <si>
-    <t>R16, R21</t>
+    <t>R14, R20</t>
   </si>
   <si>
     <t>603-RT0603FRD07100KL</t>
   </si>
   <si>
-    <t>RC0603FR-100RL</t>
-  </si>
-  <si>
-    <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0603, 0Ohms, 1%, 1/10W</t>
+    <t>RT0603DRD07330KL</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors - SMD 330K OHM .5% 25PPM 1/10W</t>
+  </si>
+  <si>
+    <t>R16</t>
+  </si>
+  <si>
+    <t>603-RT0603DRD07330KL</t>
+  </si>
+  <si>
+    <t>RT0603FRE0710KL</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors - SMD 10K ohm 1% 1/10W</t>
   </si>
   <si>
     <t>R17</t>
   </si>
   <si>
-    <t>RC0603FR-10100RL</t>
-  </si>
-  <si>
-    <t>603-RC0603FR-10100RL</t>
-  </si>
-  <si>
-    <t>RT0603FRE0710KL</t>
-  </si>
-  <si>
-    <t>Thin Film Resistors - SMD 10K ohm 1% 1/10W</t>
+    <t>603-RT0603FRE0710KL</t>
+  </si>
+  <si>
+    <t>RT0603BRD07120KL</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors - SMD 1/10W 120K ohm .1% 25ppm</t>
+  </si>
+  <si>
+    <t>R18</t>
+  </si>
+  <si>
+    <t>603-RT0603BRD07120KL</t>
+  </si>
+  <si>
+    <t>RT0805BRD07732KL</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors - SMD 732 kOhms 25PPM/C 125mW 0805 10%</t>
   </si>
   <si>
     <t>R19</t>
   </si>
   <si>
-    <t>603-RT0603FRE0710KL</t>
+    <t>603-RT0805BRD07732KL</t>
   </si>
   <si>
     <t>RC0603FR-07470RL</t>
@@ -476,21 +509,21 @@
     <t>470 Ohms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Moisture Resistant Thick Film</t>
   </si>
   <si>
+    <t>R21</t>
+  </si>
+  <si>
+    <t>603-RC0603FR-07470RL</t>
+  </si>
+  <si>
+    <t>RT0603DRD072KL</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors - SMD 2K Ohm 0.5% 1/10W 75 Volts 25ppm</t>
+  </si>
+  <si>
     <t>R22</t>
   </si>
   <si>
-    <t>603-RC0603FR-07470RL</t>
-  </si>
-  <si>
-    <t>RT0603DRD072KL</t>
-  </si>
-  <si>
-    <t>Thin Film Resistors - SMD 2K Ohm 0.5% 1/10W 75 Volts 25ppm</t>
-  </si>
-  <si>
-    <t>R23</t>
-  </si>
-  <si>
     <t>603-RT0603DRD072KL</t>
   </si>
   <si>
@@ -500,7 +533,7 @@
     <t>Thick Film Resistors - SMD 0 Ohms 250 mW 1206 1%</t>
   </si>
   <si>
-    <t>R24, R25, R26, R27, R28, R29, R30, R31, R32</t>
+    <t>R23, R24, R25, R26, R27, R28, R29, R30, R31</t>
   </si>
   <si>
     <t>603-RC1206FR-070RL</t>
@@ -579,6 +612,9 @@
   </si>
   <si>
     <t>S-8261AAXMD-G2XT2U</t>
+  </si>
+  <si>
+    <t>Battery Battery Protection IC Lithium Ion/Polymer SOT-23-6</t>
   </si>
   <si>
     <t>U5</t>
@@ -978,8 +1014,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58A796BB-D75D-480F-BEBC-B9239CFAA2C9}">
-  <dimension ref="A1:M39"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2D8B179-39A7-4591-857E-C79B8393CF1B}">
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" customWidth="1"/>
@@ -1129,7 +1165,7 @@
         <v>27</v>
       </c>
       <c r="F4" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>17</v>
@@ -1207,10 +1243,10 @@
         <v>35</v>
       </c>
       <c r="F6" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>33</v>
@@ -1222,13 +1258,13 @@
         <v>19</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L6" s="1">
-        <v>0.56999999999999995</v>
+        <v>0.11</v>
       </c>
       <c r="M6" s="1">
-        <v>1.1399999999999999</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -1236,38 +1272,38 @@
         <v>13</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="F7" s="1">
         <v>2</v>
       </c>
       <c r="G7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="L7" s="1">
-        <v>1.25</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="M7" s="1">
-        <v>2.5</v>
+        <v>1.1399999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -1275,38 +1311,38 @@
         <v>13</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" s="1">
+        <v>2</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F8" s="1">
-        <v>1</v>
-      </c>
-      <c r="G8" s="2" t="s">
+      <c r="I8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>48</v>
-      </c>
       <c r="L8" s="1">
-        <v>3.14</v>
+        <v>1.25</v>
       </c>
       <c r="M8" s="1">
-        <v>3.14</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -1314,38 +1350,38 @@
         <v>13</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="1">
+        <v>1</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="1">
-        <v>1</v>
-      </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K9" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="L9" s="1">
-        <v>0.17</v>
+        <v>3.14</v>
       </c>
       <c r="M9" s="1">
-        <v>0.17</v>
+        <v>3.14</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -1353,38 +1389,38 @@
         <v>13</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="1">
+        <v>1</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F10" s="1">
-        <v>1</v>
-      </c>
-      <c r="G10" s="2" t="s">
+      <c r="I10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K10" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H10" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="L10" s="1">
-        <v>1.05</v>
+        <v>0.17</v>
       </c>
       <c r="M10" s="1">
-        <v>1.05</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -1392,38 +1428,38 @@
         <v>13</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="1">
+        <v>1</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F11" s="1">
-        <v>2</v>
-      </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K11" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="H11" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>64</v>
-      </c>
       <c r="L11" s="1">
-        <v>0.32</v>
+        <v>1.05</v>
       </c>
       <c r="M11" s="1">
-        <v>0.64</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -1431,38 +1467,38 @@
         <v>13</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="2" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>66</v>
       </c>
       <c r="F12" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>67</v>
       </c>
       <c r="H12" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K12" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="I12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="L12" s="1">
-        <v>0.2</v>
+        <v>0.32</v>
       </c>
       <c r="M12" s="1">
-        <v>0.8</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -1470,38 +1506,38 @@
         <v>13</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="1">
+        <v>4</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F13" s="1">
-        <v>2</v>
-      </c>
-      <c r="G13" s="2" t="s">
+      <c r="H13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K13" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="H13" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="L13" s="1">
-        <v>4.3899999999999997</v>
+        <v>0.1</v>
       </c>
       <c r="M13" s="1">
-        <v>8.7799999999999994</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
@@ -1509,23 +1545,23 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" s="1">
+        <v>2</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="H14" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="F14" s="1">
-        <v>1</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>18</v>
@@ -1537,10 +1573,10 @@
         <v>79</v>
       </c>
       <c r="L14" s="1">
-        <v>0.78</v>
+        <v>4.3899999999999997</v>
       </c>
       <c r="M14" s="1">
-        <v>0.78</v>
+        <v>8.7799999999999994</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -1561,7 +1597,7 @@
         <v>1</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>17</v>
+        <v>62</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>80</v>
@@ -1576,10 +1612,10 @@
         <v>83</v>
       </c>
       <c r="L15" s="1">
-        <v>0.1</v>
+        <v>0.78</v>
       </c>
       <c r="M15" s="1">
-        <v>0.1</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -1681,16 +1717,16 @@
         <v>17</v>
       </c>
       <c r="H18" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K18" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="L18" s="1">
         <v>0.1</v>
@@ -1704,38 +1740,38 @@
         <v>13</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>99</v>
-      </c>
       <c r="F19" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>17</v>
       </c>
       <c r="H19" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K19" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="I19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>101</v>
-      </c>
       <c r="L19" s="1">
-        <v>2.3E-2</v>
+        <v>0.1</v>
       </c>
       <c r="M19" s="1">
-        <v>0.23</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -1743,23 +1779,23 @@
         <v>13</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="F20" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>17</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>18</v>
@@ -1771,10 +1807,10 @@
         <v>105</v>
       </c>
       <c r="L20" s="1">
-        <v>0.1</v>
+        <v>2.3E-2</v>
       </c>
       <c r="M20" s="1">
-        <v>0.1</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -1792,7 +1828,7 @@
         <v>108</v>
       </c>
       <c r="F21" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>17</v>
@@ -1810,10 +1846,10 @@
         <v>109</v>
       </c>
       <c r="L21" s="1">
-        <v>1.2999999999999999E-2</v>
+        <v>0.1</v>
       </c>
       <c r="M21" s="1">
-        <v>0.13</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -1831,7 +1867,7 @@
         <v>112</v>
       </c>
       <c r="F22" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>17</v>
@@ -1849,10 +1885,10 @@
         <v>113</v>
       </c>
       <c r="L22" s="1">
-        <v>0.1</v>
+        <v>1.2999999999999999E-2</v>
       </c>
       <c r="M22" s="1">
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
@@ -1948,7 +1984,7 @@
         <v>124</v>
       </c>
       <c r="F25" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>17</v>
@@ -1966,10 +2002,10 @@
         <v>125</v>
       </c>
       <c r="L25" s="1">
-        <v>1.0999999999999999E-2</v>
+        <v>0.1</v>
       </c>
       <c r="M25" s="1">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
@@ -1987,7 +2023,7 @@
         <v>128</v>
       </c>
       <c r="F26" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>17</v>
@@ -2008,7 +2044,7 @@
         <v>0.1</v>
       </c>
       <c r="M26" s="1">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
@@ -2026,7 +2062,7 @@
         <v>132</v>
       </c>
       <c r="F27" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>17</v>
@@ -2047,7 +2083,7 @@
         <v>0.1</v>
       </c>
       <c r="M27" s="1">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
@@ -2065,28 +2101,28 @@
         <v>136</v>
       </c>
       <c r="F28" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>17</v>
       </c>
       <c r="H28" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K28" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="I28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>138</v>
-      </c>
       <c r="L28" s="1">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="M28" s="1">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
@@ -2094,14 +2130,14 @@
         <v>13</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="F29" s="1">
         <v>1</v>
@@ -2110,7 +2146,7 @@
         <v>17</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>18</v>
@@ -2119,7 +2155,7 @@
         <v>19</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="L29" s="1">
         <v>0.1</v>
@@ -2133,14 +2169,14 @@
         <v>13</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C30" s="1"/>
       <c r="D30" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>144</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>145</v>
       </c>
       <c r="F30" s="1">
         <v>1</v>
@@ -2149,7 +2185,7 @@
         <v>17</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>18</v>
@@ -2158,13 +2194,13 @@
         <v>19</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L30" s="1">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="M30" s="1">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
@@ -2172,14 +2208,14 @@
         <v>13</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>149</v>
       </c>
       <c r="F31" s="1">
         <v>1</v>
@@ -2188,7 +2224,7 @@
         <v>17</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>18</v>
@@ -2197,7 +2233,7 @@
         <v>19</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="L31" s="1">
         <v>0.1</v>
@@ -2211,23 +2247,23 @@
         <v>13</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C32" s="1"/>
       <c r="D32" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>153</v>
-      </c>
       <c r="F32" s="1">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>17</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I32" s="2" t="s">
         <v>18</v>
@@ -2236,13 +2272,13 @@
         <v>19</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="L32" s="1">
-        <v>0.02</v>
+        <v>0.1</v>
       </c>
       <c r="M32" s="1">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
@@ -2250,38 +2286,38 @@
         <v>13</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C33" s="1"/>
       <c r="D33" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="F33" s="1">
+        <v>1</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K33" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="F33" s="1">
-        <v>1</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="I33" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K33" s="2" t="s">
-        <v>159</v>
-      </c>
       <c r="L33" s="1">
-        <v>0.57999999999999996</v>
+        <v>0.15</v>
       </c>
       <c r="M33" s="1">
-        <v>0.57999999999999996</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
@@ -2289,38 +2325,38 @@
         <v>13</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="F34" s="1">
+        <v>1</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K34" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="F34" s="1">
-        <v>1</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="I34" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J34" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>164</v>
-      </c>
       <c r="L34" s="1">
-        <v>0.77</v>
+        <v>0.1</v>
       </c>
       <c r="M34" s="1">
-        <v>0.77</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
@@ -2328,38 +2364,38 @@
         <v>13</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="2" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F35" s="1">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
       <c r="H35" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K35" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="I35" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>169</v>
-      </c>
       <c r="L35" s="1">
-        <v>3.07</v>
+        <v>0.02</v>
       </c>
       <c r="M35" s="1">
-        <v>3.07</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
@@ -2367,38 +2403,38 @@
         <v>13</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="F36" s="1">
         <v>1</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="H36" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K36" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="I36" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>174</v>
-      </c>
       <c r="L36" s="1">
-        <v>3.86</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="M36" s="1">
-        <v>3.86</v>
+        <v>0.57999999999999996</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
@@ -2406,38 +2442,38 @@
         <v>13</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="2" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="F37" s="1">
         <v>1</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="H37" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K37" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="I37" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>178</v>
-      </c>
       <c r="L37" s="1">
-        <v>2.15</v>
+        <v>0.77</v>
       </c>
       <c r="M37" s="1">
-        <v>2.15</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
@@ -2445,38 +2481,38 @@
         <v>13</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="2" t="s">
-        <v>13</v>
+        <v>177</v>
       </c>
       <c r="E38" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F38" s="1">
+        <v>1</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K38" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="F38" s="1">
-        <v>1</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="I38" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J38" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K38" s="2" t="s">
-        <v>182</v>
-      </c>
       <c r="L38" s="1">
-        <v>0.98</v>
+        <v>3.07</v>
       </c>
       <c r="M38" s="1">
-        <v>0.98</v>
+        <v>3.07</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
@@ -2484,37 +2520,154 @@
         <v>13</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C39" s="1"/>
       <c r="D39" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="F39" s="1">
+        <v>1</v>
+      </c>
+      <c r="G39" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="E39" s="2" t="s">
+      <c r="H39" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K39" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="F39" s="1">
-        <v>1</v>
-      </c>
-      <c r="G39" s="2" t="s">
+      <c r="L39" s="1">
+        <v>3.52</v>
+      </c>
+      <c r="M39" s="1">
+        <v>3.52</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="H39" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="I39" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J39" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K39" s="2" t="s">
+      <c r="C40" s="1"/>
+      <c r="D40" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="L39" s="1">
+      <c r="E40" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F40" s="1">
+        <v>1</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="L40" s="1">
+        <v>2.15</v>
+      </c>
+      <c r="M40" s="1">
+        <v>2.15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C41" s="1"/>
+      <c r="D41" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="F41" s="1">
+        <v>1</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="L41" s="1">
+        <v>0.98</v>
+      </c>
+      <c r="M41" s="1">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C42" s="1"/>
+      <c r="D42" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F42" s="1">
+        <v>1</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="L42" s="1">
         <v>0.45</v>
       </c>
-      <c r="M39" s="1">
+      <c r="M42" s="1">
         <v>0.45</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update output files and board shape
</commit_message>
<xml_diff>
--- a/Project Ouputs/BOM/Bill of Materials-sme-pcb-energysolution-s01.xlsx
+++ b/Project Ouputs/BOM/Bill of Materials-sme-pcb-energysolution-s01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\sme\PCB\sme-pcb-energysolution-s01\Project Ouputs\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{046D59B9-3DED-43CA-ABD9-52294A7AE2A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D3ADFCD1-6DFD-407D-B580-EB3C26E7FC4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C15F647B-C887-43F2-9E13-23750635C920}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{54805E00-C042-4EC0-A81B-DC3E5BA326E8}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-sme-pcb-energ" sheetId="1" r:id="rId1"/>
@@ -1014,7 +1014,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2D8B179-39A7-4591-857E-C79B8393CF1B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E883881-AD70-46E2-9CE5-C05C65F180A6}">
   <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>